<commit_message>
Add Excel file opening feature
</commit_message>
<xml_diff>
--- a/transactions.xlsx
+++ b/transactions.xlsx
@@ -1,56 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:a15="http://schemas.microsoft.com/office/drawing/2012/main" xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:co="http://ncloudtech.com" xmlns:co-ooxml="http://ncloudtech.com/ooxml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:s="http://schemas.openxmlformats.org/officeDocument/2006/sharedTypes" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main" xmlns:w10="urn:schemas-microsoft-com:office:word" xmlns:w14="http://schemas.microsoft.com/office/word/2010/wordml" xmlns:w15="http://schemas.microsoft.com/office/word/2012/wordml" xmlns:wp="http://schemas.openxmlformats.org/drawingml/2006/wordprocessingDrawing" xmlns:wpg="http://schemas.microsoft.com/office/word/2010/wordprocessingGroup" xmlns:wps="http://schemas.microsoft.com/office/word/2010/wordprocessingShape" xmlns:x="urn:schemas-microsoft-com:office:excel" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" mc:Ignorable="co co-ooxml w14 x14 w15">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="9302"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <sheets>
-    <sheet name="История" r:id="rId1" sheetId="1" state="visible"/>
+    <sheet name="История" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:a15="http://schemas.microsoft.com/office/drawing/2012/main" xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:co="http://ncloudtech.com" xmlns:co-ooxml="http://ncloudtech.com/ooxml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:s="http://schemas.openxmlformats.org/officeDocument/2006/sharedTypes" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main" xmlns:w10="urn:schemas-microsoft-com:office:word" xmlns:w14="http://schemas.microsoft.com/office/word/2010/wordml" xmlns:w15="http://schemas.microsoft.com/office/word/2012/wordml" xmlns:wp="http://schemas.openxmlformats.org/drawingml/2006/wordprocessingDrawing" xmlns:wpg="http://schemas.microsoft.com/office/word/2010/wordprocessingGroup" xmlns:wps="http://schemas.microsoft.com/office/word/2010/wordprocessingShape" xmlns:x="urn:schemas-microsoft-com:office:excel" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" mc:Ignorable="co co-ooxml w14 x14 w15">
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>Дата</t>
-  </si>
-  <si>
-    <t>Итог за день (UZS)</t>
-  </si>
-  <si>
-    <t>2026-10-21</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:a15="http://schemas.microsoft.com/office/drawing/2012/main" xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:co="http://ncloudtech.com" xmlns:co-ooxml="http://ncloudtech.com/ooxml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:s="http://schemas.openxmlformats.org/officeDocument/2006/sharedTypes" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main" xmlns:w10="urn:schemas-microsoft-com:office:word" xmlns:w14="http://schemas.microsoft.com/office/word/2010/wordml" xmlns:w15="http://schemas.microsoft.com/office/word/2012/wordml" xmlns:wp="http://schemas.openxmlformats.org/drawingml/2006/wordprocessingDrawing" xmlns:wpg="http://schemas.microsoft.com/office/word/2010/wordprocessingGroup" xmlns:wps="http://schemas.microsoft.com/office/word/2010/wordprocessingShape" xmlns:x="urn:schemas-microsoft-com:office:excel" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" mc:Ignorable="co co-ooxml w14 x14 w15">
-  <numFmts>
-    <numFmt co:extendedFormatCode="General" formatCode="General" numFmtId="1000"/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
-      <color theme="1" tint="0"/>
+      <color theme="1"/>
       <sz val="11"/>
     </font>
     <font>
-      <color theme="1" tint="0"/>
+      <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="true"/>
+      <b val="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -58,25 +39,95 @@
   </fills>
   <borders count="1">
     <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf applyFont="true" applyNumberFormat="true" borderId="0" fillId="0" fontId="1" numFmtId="1000" quotePrefix="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf applyFont="true" applyNumberFormat="true" borderId="0" fillId="0" fontId="1" numFmtId="1000" quotePrefix="false"/>
-    <xf applyFont="true" applyNumberFormat="true" borderId="0" fillId="0" fontId="2" numFmtId="1000" quotePrefix="false"/>
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle builtinId="0" name="Normal" xfId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultPivotStyle="PivotStyleMedium4" defaultTableStyle="TableStyleMedium9"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -285,41 +336,63 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:a15="http://schemas.microsoft.com/office/drawing/2012/main" xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:co="http://ncloudtech.com" xmlns:co-ooxml="http://ncloudtech.com/ooxml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:s="http://schemas.openxmlformats.org/officeDocument/2006/sharedTypes" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main" xmlns:w10="urn:schemas-microsoft-com:office:word" xmlns:w14="http://schemas.microsoft.com/office/word/2010/wordml" xmlns:w15="http://schemas.microsoft.com/office/word/2012/wordml" xmlns:wp="http://schemas.openxmlformats.org/drawingml/2006/wordprocessingDrawing" xmlns:wpg="http://schemas.microsoft.com/office/word/2010/wordprocessingGroup" xmlns:wps="http://schemas.microsoft.com/office/word/2010/wordprocessingShape" xmlns:x="urn:schemas-microsoft-com:office:excel" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" mc:Ignorable="co co-ooxml w14 x14 w15">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="true" summaryRight="true"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr baseColWidth="8" customHeight="false" defaultColWidth="9.14062530925693" defaultRowHeight="15" zeroHeight="false"/>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625309256929" defaultRowHeight="15" customHeight="0" zeroHeight="0"/>
   <cols>
-    <col customWidth="true" max="1" min="1" outlineLevel="0" width="10.0000003383324"/>
-    <col customWidth="true" max="2" min="2" outlineLevel="0" width="16"/>
-    <col customWidth="true" max="3" min="3" outlineLevel="0" width="25.0000008458309"/>
+    <col width="10.0000003383324" customWidth="1" style="2" min="1" max="1"/>
+    <col width="16" customWidth="1" style="2" min="2" max="2"/>
+    <col width="25.0000008458309" customWidth="1" style="2" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row outlineLevel="0" r="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1" s="2">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Дата</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Итог за день (UZS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" s="2">
+      <c r="A2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-    </row>
-    <row outlineLevel="0" r="2">
-      <c r="A2" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="0" t="n">
-        <v>400000</v>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>-50000</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>